<commit_message>
Tablas_Stock archivo - Sep-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock_2026_09.xlsx
+++ b/Tablas/Tablas_Stock_2026_09.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Satisfaccion global 69% (+0pp vs agosto). 681 respuestas, tasa 23% sobre cumplidos. ALUMBRADO 78%, RESIDUOS y TRANSITO 73%; ARBOLADO 10% (2 de 20) es la peor del municipio y CTRL ACTIVIDADES 31% mantiene la brecha con su cierre. CALLES y TRANSITO con muestra insuficiente.</t>
+          <t>Satisfaccion global 69% (+0pp vs agosto). 681 respuestas, tasa 23% sobre cumplidos. ALUMBRADO 78%, RESIDUOS y TRANSITO 73%; ARBOLADO 10% (2 de 20) es la peor del municipio y CTRL ACTIVIDADES 31% mantiene la brecha con su cierre. CALLES 57% (21 respuestas) y CTRL ESPACIO 48%.</t>
         </is>
       </c>
     </row>
@@ -623,7 +623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -726,7 +726,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Cierre del area 20%-&gt;15% (Ago-2026 a Sep-2026), séptimo mes en zona crítica. Cancelado 7% sobre cerrados; 399 casos sin cerrar.</t>
+          <t>Cierre del area 20%-&gt;15% (Ago-2026 a Sep-2026), séptimo mes en zona crítica desde Mar-2026. Cancelado 7% sobre cerrados; 399 casos sin cerrar.</t>
         </is>
       </c>
     </row>
@@ -812,49 +812,49 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo - Cable cortado</t>
+          <t>Cierre bajo (area)</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>117 casos, 1% cierre</t>
+          <t>39%</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Cable cortado: 117 casos en Sep-2026 (77 en Ago-2026), cierre 12%-&gt;1%. Sigue con cierre bajo.</t>
+          <t>Cierre del area 39% en Sep-2026 (125 de 318), en zona crítica desde Sep-2026. Arrastra desde Ago-2026 el cierre bajo de Cable cortado (77-&gt;117 casos, cierre 12%-&gt;1%) y Poste en mal estado/sin mantenimiento (24-&gt;21 casos, cierre 22%-&gt;14%); se suma Reparación de vereda rota por empresa de servicio (27 casos, 15% de cierre). Cancelado 2% sobre cerrados.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>PERSISTE</t>
+          <t>NUEVA</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Ago-2026</t>
+          <t>Sep-2026</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo - Poste en mal estado/sin mantenimiento</t>
+          <t>Cancelado alto en cerrados</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>21 casos, 14% cierre</t>
+          <t>11% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Poste en mal estado/sin mantenimiento: 21 casos en Sep-2026 (24 en Ago-2026), cierre 22%-&gt;14%. Sigue con cierre bajo.</t>
+          <t>11% de los cerrados de Sep-2026 son Cancelados (8 de 74, donut Cierres por Estado): Reparación o daño de caniles en parque/plaza (5 de 7 cierres) y Inconvenientes con intervenciones de arbolado (3 de 33 cierres). Revisar la calidad de esos cierres.</t>
         </is>
       </c>
     </row>
@@ -876,17 +876,17 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Cancelado alto en cerrados</t>
+          <t>Suba de volumen - Árbol obstruye luminaria</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>11% (sobre cerrados)</t>
+          <t>11-&gt;38 (+245%)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>11% de los cerrados de Sep-2026 son Cancelados (8 de 74, donut Cierres por Estado): Reparación o daño de caniles en parque/plaza (5 de 7 cierres) y Inconvenientes con intervenciones de arbolado (3 de 33 cierres). Revisar la calidad de esos cierres.</t>
+          <t>Árbol obstruye luminaria: 11 casos en Ago-2026 a 38 en Sep-2026 (+245%), maximo de los ultimos 13 meses; 11% de cierre.</t>
         </is>
       </c>
     </row>
@@ -903,22 +903,22 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Calles y Veredas</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Suba de volumen - Árbol obstruye luminaria</t>
+          <t>SLA critico (area)</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>11-&gt;38 (+245%)</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Árbol obstruye luminaria: 11 casos en Ago-2026 a 38 en Sep-2026 (+245%), maximo de los ultimos 13 meses; 11% de cierre.</t>
+          <t>SLA del area 28% en Sep-2026: 51 de los 71 cierres fuera del plazo por tipo. Tiempo promedio 10 dias.</t>
         </is>
       </c>
     </row>
@@ -940,17 +940,17 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>SLA critico (area)</t>
+          <t>Cancelado alto en cerrados</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>7% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>SLA del area 28% en Sep-2026: 51 de los 71 cierres fuera del plazo por tipo. Tiempo promedio 10 dias.</t>
+          <t>7% de los cerrados de Sep-2026 son Cancelados (5 de 71, donut Cierres por Estado): Bache en calle de asfalto (2 de 42 cierres) y Repintado / reparación de demarcación vial en calle o cordón (1 de 4 cierres). Revisar la calidad de esos cierres.</t>
         </is>
       </c>
     </row>
@@ -972,17 +972,17 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Cancelado alto en cerrados</t>
+          <t>Suba de volumen - Reparación/construcción de cordón</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>7% (sobre cerrados)</t>
+          <t>69-&gt;111 (+61%)</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>7% de los cerrados de Sep-2026 son Cancelados (5 de 71, donut Cierres por Estado): Bache en calle de asfalto (2 de 42 cierres) y Repintado / reparación de demarcación vial en calle o cordón (1 de 4 cierres). Revisar la calidad de esos cierres.</t>
+          <t>Reparación/construcción de cordón: 69 casos en Ago-2026 a 111 en Sep-2026 (+61%), maximo de los ultimos 13 meses; 5% de cierre.</t>
         </is>
       </c>
     </row>
@@ -1004,17 +1004,17 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Suba de volumen - Reparación/construcción de cordón</t>
+          <t>Suba de volumen - Reparación de rampa de accesibilidad</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>69-&gt;111 (+61%)</t>
+          <t>15-&gt;36 (+140%)</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Reparación/construcción de cordón: 69 casos en Ago-2026 a 111 en Sep-2026 (+61%), maximo de los ultimos 13 meses; 5% de cierre.</t>
+          <t>Reparación de rampa de accesibilidad: 15 casos en Ago-2026 a 36 en Sep-2026 (+140%), maximo de los ultimos 13 meses; 6% de cierre.</t>
         </is>
       </c>
     </row>
@@ -1036,17 +1036,17 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Suba de volumen - Reparación de rampa de accesibilidad</t>
+          <t>Volumen anomalo - Construcción de cuneta</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>15-&gt;36 (+140%)</t>
+          <t>4-&gt;22</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Reparación de rampa de accesibilidad: 15 casos en Ago-2026 a 36 en Sep-2026 (+140%), maximo de los ultimos 13 meses; 6% de cierre.</t>
+          <t>Construcción de cuneta: pasa de 4 casos en Ago-2026 a 22 en Sep-2026, maximo de los ultimos 13 meses sobre una base historica baja; ningún cierre.</t>
         </is>
       </c>
     </row>
@@ -1063,22 +1063,22 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Volumen anomalo - Construcción de cuneta</t>
+          <t>Suba de volumen - Reparación de vereda rota por empresa de servicio</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>4-&gt;22</t>
+          <t>19-&gt;27 (+42%)</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Construcción de cuneta: pasa de 4 casos en Ago-2026 a 22 en Sep-2026, maximo de los ultimos 13 meses sobre una base historica baja; ningún cierre.</t>
+          <t>Reparación de vereda rota por empresa de servicio: 19 casos en Ago-2026 a 27 en Sep-2026 (+42%), maximo de los ultimos 13 meses; 15% de cierre.</t>
         </is>
       </c>
     </row>
@@ -1095,84 +1095,20 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Transito</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo (area)</t>
+          <t>Cancelado alto en cerrados</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>3% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>Cierre del area 39% en Sep-2026 (125 de 318). Lo arrastra: Cable cortado 117 casos (1% de cierre); Reparación de vereda rota por empresa de servicio 27 casos (15% de cierre). Cancelado 2% sobre cerrados.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>Sep-2026</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Control del Espacio Publico</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
-        <is>
-          <t>Suba de volumen - Reparación de vereda rota por empresa de servicio</t>
-        </is>
-      </c>
-      <c r="E16" s="3" t="inlineStr">
-        <is>
-          <t>19-&gt;27 (+42%)</t>
-        </is>
-      </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>Reparación de vereda rota por empresa de servicio: 19 casos en Ago-2026 a 27 en Sep-2026 (+42%), maximo de los ultimos 13 meses; 15% de cierre.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>NUEVA</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>Sep-2026</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Cancelado alto en cerrados</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>3% (sobre cerrados)</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>3% de los cerrados de Sep-2026 son Cancelados (13 de 372, donut Cierres por Estado): Vehículos Abandonados (10 de 320 cierres) y Reparación de semáforo (3 de 40 cierres). Revisar la calidad de esos cierres.</t>
         </is>

</xml_diff>